<commit_message>
Update Realisasi 23 Oktober 25
Update Realisasi 23 Oktober 25
</commit_message>
<xml_diff>
--- a/Database/MONITORING DETAIL TRANSAKSI FA 16 SEGMEN VERSI SP2D.xlsx
+++ b/Database/MONITORING DETAIL TRANSAKSI FA 16 SEGMEN VERSI SP2D.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1502">
   <si>
     <t>MONITORING DETAIL TRANSAKSI FA 16 SEGMEN VERSI SP2D</t>
   </si>
@@ -4352,6 +4352,27 @@
     <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan September 2025 untuk 1 Pegawai/2 Jiwa</t>
   </si>
   <si>
+    <t>2025-10-17</t>
+  </si>
+  <si>
+    <t>'00419T</t>
+  </si>
+  <si>
+    <t>'259991310815027</t>
+  </si>
+  <si>
+    <t>Pembayaran belanja barang berupa tagihan telepon bulan Oktober 2025 untuk 12 invoice</t>
+  </si>
+  <si>
+    <t>'00420T</t>
+  </si>
+  <si>
+    <t>'259991320454564</t>
+  </si>
+  <si>
+    <t>Pembayaran belanja barang berupa tagihan listrik bulan Oktober 2025 untuk 6 invoice</t>
+  </si>
+  <si>
     <t>'00421T</t>
   </si>
   <si>
@@ -4413,6 +4434,93 @@
   </si>
   <si>
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan September 2025 untuk 5 Pegawai</t>
+  </si>
+  <si>
+    <t>2025-10-16</t>
+  </si>
+  <si>
+    <t>'00437T</t>
+  </si>
+  <si>
+    <t>'259991320487988</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang berupa Tagihan Internet Bulan September 2025 idpel No.GO18A106 An Balai Riset Perikanan Budidaya Air Tawar dan Penyuluhan Perikanan</t>
+  </si>
+  <si>
+    <t>'00438T</t>
+  </si>
+  <si>
+    <t>'259991330302342</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan September tahun 2025 untuk 169 Pegawai</t>
+  </si>
+  <si>
+    <t>'00439T</t>
+  </si>
+  <si>
+    <t>'259991310881244</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan September tahun 2025 untuk 131 Pegawai</t>
+  </si>
+  <si>
+    <t>'00440T</t>
+  </si>
+  <si>
+    <t>'259991310881247</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan September 2025 untuk 34 Pegawai</t>
+  </si>
+  <si>
+    <t>'00441T</t>
+  </si>
+  <si>
+    <t>'259991310881245</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan September tahun 2025 untuk 50 Pegawai</t>
+  </si>
+  <si>
+    <t>'00442T</t>
+  </si>
+  <si>
+    <t>'259991330302343</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan September tahun 2025 untuk 63 Pegawai</t>
+  </si>
+  <si>
+    <t>'00443T</t>
+  </si>
+  <si>
+    <t>'259991310881246</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan September tahun 2025 untuk 35 Pegawai</t>
+  </si>
+  <si>
+    <t>'00444T</t>
+  </si>
+  <si>
+    <t>'259991330302344</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan September tahun 2025 untuk 23 Pegawai</t>
+  </si>
+  <si>
+    <t>2025-10-21</t>
+  </si>
+  <si>
+    <t>'00445T</t>
+  </si>
+  <si>
+    <t>'259991310895627</t>
+  </si>
+  <si>
+    <t>'403829.023.521811.03212WA.2378EBA.A000000001.00000.2.0252.2.000000.000000.994.002.DA.000292</t>
   </si>
 </sst>
 </file>
@@ -4755,7 +4863,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:L1464"/>
+  <dimension ref="A1:L1478"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -59685,19 +59793,19 @@
         <v>13</v>
       </c>
       <c r="D1448" t="s">
-        <v>1433</v>
+        <v>1445</v>
       </c>
       <c r="E1448" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="F1448" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
       <c r="G1448" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
       <c r="H1448" t="s">
-        <v>233</v>
+        <v>83</v>
       </c>
       <c r="I1448" t="s">
         <v>19</v>
@@ -59706,10 +59814,10 @@
         <v>1</v>
       </c>
       <c r="K1448">
-        <v>7105000</v>
+        <v>266844</v>
       </c>
       <c r="L1448">
-        <v>7105000</v>
+        <v>266844</v>
       </c>
     </row>
     <row r="1449" spans="1:12">
@@ -59723,19 +59831,19 @@
         <v>13</v>
       </c>
       <c r="D1449" t="s">
-        <v>1433</v>
+        <v>1445</v>
       </c>
       <c r="E1449" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="F1449" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
       <c r="G1449" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
       <c r="H1449" t="s">
-        <v>234</v>
+        <v>84</v>
       </c>
       <c r="I1449" t="s">
         <v>19</v>
@@ -59744,10 +59852,10 @@
         <v>1</v>
       </c>
       <c r="K1449">
-        <v>30636000</v>
+        <v>2580750</v>
       </c>
       <c r="L1449">
-        <v>30636000</v>
+        <v>2580750</v>
       </c>
     </row>
     <row r="1450" spans="1:12">
@@ -59761,19 +59869,19 @@
         <v>13</v>
       </c>
       <c r="D1450" t="s">
-        <v>1433</v>
+        <v>1445</v>
       </c>
       <c r="E1450" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
       <c r="F1450" t="s">
-        <v>1449</v>
+        <v>1450</v>
       </c>
       <c r="G1450" t="s">
-        <v>1450</v>
+        <v>1451</v>
       </c>
       <c r="H1450" t="s">
-        <v>233</v>
+        <v>79</v>
       </c>
       <c r="I1450" t="s">
         <v>19</v>
@@ -59782,10 +59890,10 @@
         <v>1</v>
       </c>
       <c r="K1450">
-        <v>1470000</v>
+        <v>39011162</v>
       </c>
       <c r="L1450">
-        <v>1470000</v>
+        <v>39011162</v>
       </c>
     </row>
     <row r="1451" spans="1:12">
@@ -59802,16 +59910,16 @@
         <v>1433</v>
       </c>
       <c r="E1451" t="s">
-        <v>1448</v>
+        <v>1452</v>
       </c>
       <c r="F1451" t="s">
-        <v>1449</v>
+        <v>1453</v>
       </c>
       <c r="G1451" t="s">
-        <v>1450</v>
+        <v>1454</v>
       </c>
       <c r="H1451" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I1451" t="s">
         <v>19</v>
@@ -59820,10 +59928,10 @@
         <v>1</v>
       </c>
       <c r="K1451">
-        <v>45843000</v>
+        <v>7105000</v>
       </c>
       <c r="L1451">
-        <v>45843000</v>
+        <v>7105000</v>
       </c>
     </row>
     <row r="1452" spans="1:12">
@@ -59840,16 +59948,16 @@
         <v>1433</v>
       </c>
       <c r="E1452" t="s">
-        <v>1451</v>
+        <v>1452</v>
       </c>
       <c r="F1452" t="s">
-        <v>1452</v>
+        <v>1453</v>
       </c>
       <c r="G1452" t="s">
-        <v>1453</v>
+        <v>1454</v>
       </c>
       <c r="H1452" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="I1452" t="s">
         <v>19</v>
@@ -59858,10 +59966,10 @@
         <v>1</v>
       </c>
       <c r="K1452">
-        <v>2170000</v>
+        <v>30636000</v>
       </c>
       <c r="L1452">
-        <v>2170000</v>
+        <v>30636000</v>
       </c>
     </row>
     <row r="1453" spans="1:12">
@@ -59878,16 +59986,16 @@
         <v>1433</v>
       </c>
       <c r="E1453" t="s">
-        <v>1451</v>
+        <v>1455</v>
       </c>
       <c r="F1453" t="s">
-        <v>1452</v>
+        <v>1456</v>
       </c>
       <c r="G1453" t="s">
-        <v>1453</v>
+        <v>1457</v>
       </c>
       <c r="H1453" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I1453" t="s">
         <v>19</v>
@@ -59896,10 +60004,10 @@
         <v>1</v>
       </c>
       <c r="K1453">
-        <v>14763000</v>
+        <v>1470000</v>
       </c>
       <c r="L1453">
-        <v>14763000</v>
+        <v>1470000</v>
       </c>
     </row>
     <row r="1454" spans="1:12">
@@ -59916,16 +60024,16 @@
         <v>1433</v>
       </c>
       <c r="E1454" t="s">
-        <v>1454</v>
+        <v>1455</v>
       </c>
       <c r="F1454" t="s">
-        <v>1455</v>
+        <v>1456</v>
       </c>
       <c r="G1454" t="s">
-        <v>1456</v>
+        <v>1457</v>
       </c>
       <c r="H1454" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="I1454" t="s">
         <v>19</v>
@@ -59934,10 +60042,10 @@
         <v>1</v>
       </c>
       <c r="K1454">
-        <v>1470000</v>
+        <v>45843000</v>
       </c>
       <c r="L1454">
-        <v>1470000</v>
+        <v>45843000</v>
       </c>
     </row>
     <row r="1455" spans="1:12">
@@ -59954,16 +60062,16 @@
         <v>1433</v>
       </c>
       <c r="E1455" t="s">
-        <v>1454</v>
+        <v>1458</v>
       </c>
       <c r="F1455" t="s">
-        <v>1455</v>
+        <v>1459</v>
       </c>
       <c r="G1455" t="s">
-        <v>1456</v>
+        <v>1460</v>
       </c>
       <c r="H1455" t="s">
-        <v>149</v>
+        <v>233</v>
       </c>
       <c r="I1455" t="s">
         <v>19</v>
@@ -59972,10 +60080,10 @@
         <v>1</v>
       </c>
       <c r="K1455">
-        <v>22829000</v>
+        <v>2170000</v>
       </c>
       <c r="L1455">
-        <v>22829000</v>
+        <v>2170000</v>
       </c>
     </row>
     <row r="1456" spans="1:12">
@@ -59992,16 +60100,16 @@
         <v>1433</v>
       </c>
       <c r="E1456" t="s">
-        <v>1454</v>
+        <v>1458</v>
       </c>
       <c r="F1456" t="s">
-        <v>1455</v>
+        <v>1459</v>
       </c>
       <c r="G1456" t="s">
-        <v>1456</v>
+        <v>1460</v>
       </c>
       <c r="H1456" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="I1456" t="s">
         <v>19</v>
@@ -60010,10 +60118,10 @@
         <v>1</v>
       </c>
       <c r="K1456">
-        <v>2419000</v>
+        <v>14763000</v>
       </c>
       <c r="L1456">
-        <v>2419000</v>
+        <v>14763000</v>
       </c>
     </row>
     <row r="1457" spans="1:12">
@@ -60030,16 +60138,16 @@
         <v>1433</v>
       </c>
       <c r="E1457" t="s">
-        <v>1457</v>
+        <v>1461</v>
       </c>
       <c r="F1457" t="s">
-        <v>1458</v>
+        <v>1462</v>
       </c>
       <c r="G1457" t="s">
-        <v>1459</v>
+        <v>1463</v>
       </c>
       <c r="H1457" t="s">
-        <v>266</v>
+        <v>241</v>
       </c>
       <c r="I1457" t="s">
         <v>19</v>
@@ -60048,10 +60156,10 @@
         <v>1</v>
       </c>
       <c r="K1457">
-        <v>10710000</v>
+        <v>1470000</v>
       </c>
       <c r="L1457">
-        <v>10710000</v>
+        <v>1470000</v>
       </c>
     </row>
     <row r="1458" spans="1:12">
@@ -60068,16 +60176,16 @@
         <v>1433</v>
       </c>
       <c r="E1458" t="s">
-        <v>1457</v>
+        <v>1461</v>
       </c>
       <c r="F1458" t="s">
-        <v>1458</v>
+        <v>1462</v>
       </c>
       <c r="G1458" t="s">
-        <v>1459</v>
+        <v>1463</v>
       </c>
       <c r="H1458" t="s">
-        <v>267</v>
+        <v>149</v>
       </c>
       <c r="I1458" t="s">
         <v>19</v>
@@ -60086,10 +60194,10 @@
         <v>1</v>
       </c>
       <c r="K1458">
-        <v>67599000</v>
+        <v>22829000</v>
       </c>
       <c r="L1458">
-        <v>67599000</v>
+        <v>22829000</v>
       </c>
     </row>
     <row r="1459" spans="1:12">
@@ -60106,16 +60214,16 @@
         <v>1433</v>
       </c>
       <c r="E1459" t="s">
-        <v>1457</v>
+        <v>1461</v>
       </c>
       <c r="F1459" t="s">
-        <v>1458</v>
+        <v>1462</v>
       </c>
       <c r="G1459" t="s">
-        <v>1459</v>
+        <v>1463</v>
       </c>
       <c r="H1459" t="s">
-        <v>268</v>
+        <v>242</v>
       </c>
       <c r="I1459" t="s">
         <v>19</v>
@@ -60124,10 +60232,10 @@
         <v>1</v>
       </c>
       <c r="K1459">
-        <v>23247000</v>
+        <v>2419000</v>
       </c>
       <c r="L1459">
-        <v>23247000</v>
+        <v>2419000</v>
       </c>
     </row>
     <row r="1460" spans="1:12">
@@ -60144,13 +60252,13 @@
         <v>1433</v>
       </c>
       <c r="E1460" t="s">
-        <v>1460</v>
+        <v>1464</v>
       </c>
       <c r="F1460" t="s">
-        <v>1461</v>
+        <v>1465</v>
       </c>
       <c r="G1460" t="s">
-        <v>1462</v>
+        <v>1466</v>
       </c>
       <c r="H1460" t="s">
         <v>266</v>
@@ -60162,10 +60270,10 @@
         <v>1</v>
       </c>
       <c r="K1460">
-        <v>10780000</v>
+        <v>10710000</v>
       </c>
       <c r="L1460">
-        <v>10780000</v>
+        <v>10710000</v>
       </c>
     </row>
     <row r="1461" spans="1:12">
@@ -60182,13 +60290,13 @@
         <v>1433</v>
       </c>
       <c r="E1461" t="s">
-        <v>1460</v>
+        <v>1464</v>
       </c>
       <c r="F1461" t="s">
-        <v>1461</v>
+        <v>1465</v>
       </c>
       <c r="G1461" t="s">
-        <v>1462</v>
+        <v>1466</v>
       </c>
       <c r="H1461" t="s">
         <v>267</v>
@@ -60200,10 +60308,10 @@
         <v>1</v>
       </c>
       <c r="K1461">
-        <v>100085000</v>
+        <v>67599000</v>
       </c>
       <c r="L1461">
-        <v>100085000</v>
+        <v>67599000</v>
       </c>
     </row>
     <row r="1462" spans="1:12">
@@ -60220,13 +60328,13 @@
         <v>1433</v>
       </c>
       <c r="E1462" t="s">
-        <v>1460</v>
+        <v>1464</v>
       </c>
       <c r="F1462" t="s">
-        <v>1461</v>
+        <v>1465</v>
       </c>
       <c r="G1462" t="s">
-        <v>1462</v>
+        <v>1466</v>
       </c>
       <c r="H1462" t="s">
         <v>268</v>
@@ -60238,10 +60346,10 @@
         <v>1</v>
       </c>
       <c r="K1462">
-        <v>20254000</v>
+        <v>23247000</v>
       </c>
       <c r="L1462">
-        <v>20254000</v>
+        <v>23247000</v>
       </c>
     </row>
     <row r="1463" spans="1:12">
@@ -60258,16 +60366,16 @@
         <v>1433</v>
       </c>
       <c r="E1463" t="s">
-        <v>1463</v>
+        <v>1467</v>
       </c>
       <c r="F1463" t="s">
-        <v>1464</v>
+        <v>1468</v>
       </c>
       <c r="G1463" t="s">
-        <v>1465</v>
+        <v>1469</v>
       </c>
       <c r="H1463" t="s">
-        <v>149</v>
+        <v>266</v>
       </c>
       <c r="I1463" t="s">
         <v>19</v>
@@ -60276,10 +60384,10 @@
         <v>1</v>
       </c>
       <c r="K1463">
-        <v>2072000</v>
+        <v>10780000</v>
       </c>
       <c r="L1463">
-        <v>2072000</v>
+        <v>10780000</v>
       </c>
     </row>
     <row r="1464" spans="1:12">
@@ -60296,28 +60404,560 @@
         <v>1433</v>
       </c>
       <c r="E1464" t="s">
+        <v>1467</v>
+      </c>
+      <c r="F1464" t="s">
+        <v>1468</v>
+      </c>
+      <c r="G1464" t="s">
+        <v>1469</v>
+      </c>
+      <c r="H1464" t="s">
+        <v>267</v>
+      </c>
+      <c r="I1464" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1464">
+        <v>1</v>
+      </c>
+      <c r="K1464">
+        <v>100085000</v>
+      </c>
+      <c r="L1464">
+        <v>100085000</v>
+      </c>
+    </row>
+    <row r="1465" spans="1:12">
+      <c r="A1465">
+        <v>1462</v>
+      </c>
+      <c r="B1465">
+        <v>403829</v>
+      </c>
+      <c r="C1465" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1465" t="s">
+        <v>1433</v>
+      </c>
+      <c r="E1465" t="s">
+        <v>1467</v>
+      </c>
+      <c r="F1465" t="s">
+        <v>1468</v>
+      </c>
+      <c r="G1465" t="s">
+        <v>1469</v>
+      </c>
+      <c r="H1465" t="s">
+        <v>268</v>
+      </c>
+      <c r="I1465" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1465">
+        <v>1</v>
+      </c>
+      <c r="K1465">
+        <v>20254000</v>
+      </c>
+      <c r="L1465">
+        <v>20254000</v>
+      </c>
+    </row>
+    <row r="1466" spans="1:12">
+      <c r="A1466">
         <v>1463</v>
       </c>
-      <c r="F1464" t="s">
+      <c r="B1466">
+        <v>403829</v>
+      </c>
+      <c r="C1466" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1466" t="s">
+        <v>1433</v>
+      </c>
+      <c r="E1466" t="s">
+        <v>1470</v>
+      </c>
+      <c r="F1466" t="s">
+        <v>1471</v>
+      </c>
+      <c r="G1466" t="s">
+        <v>1472</v>
+      </c>
+      <c r="H1466" t="s">
+        <v>149</v>
+      </c>
+      <c r="I1466" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1466">
+        <v>1</v>
+      </c>
+      <c r="K1466">
+        <v>2072000</v>
+      </c>
+      <c r="L1466">
+        <v>2072000</v>
+      </c>
+    </row>
+    <row r="1467" spans="1:12">
+      <c r="A1467">
         <v>1464</v>
       </c>
-      <c r="G1464" t="s">
+      <c r="B1467">
+        <v>403829</v>
+      </c>
+      <c r="C1467" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1467" t="s">
+        <v>1433</v>
+      </c>
+      <c r="E1467" t="s">
+        <v>1470</v>
+      </c>
+      <c r="F1467" t="s">
+        <v>1471</v>
+      </c>
+      <c r="G1467" t="s">
+        <v>1472</v>
+      </c>
+      <c r="H1467" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1467" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1467">
+        <v>1</v>
+      </c>
+      <c r="K1467">
+        <v>1722000</v>
+      </c>
+      <c r="L1467">
+        <v>1722000</v>
+      </c>
+    </row>
+    <row r="1468" spans="1:12">
+      <c r="A1468">
         <v>1465</v>
       </c>
-      <c r="H1464" t="s">
-        <v>242</v>
-      </c>
-      <c r="I1464" t="s">
-        <v>19</v>
-      </c>
-      <c r="J1464">
-        <v>1</v>
-      </c>
-      <c r="K1464">
-        <v>1722000</v>
-      </c>
-      <c r="L1464">
-        <v>1722000</v>
+      <c r="B1468">
+        <v>403829</v>
+      </c>
+      <c r="C1468" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1468" t="s">
+        <v>1473</v>
+      </c>
+      <c r="E1468" t="s">
+        <v>1474</v>
+      </c>
+      <c r="F1468" t="s">
+        <v>1475</v>
+      </c>
+      <c r="G1468" t="s">
+        <v>1476</v>
+      </c>
+      <c r="H1468" t="s">
+        <v>84</v>
+      </c>
+      <c r="I1468" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1468">
+        <v>1</v>
+      </c>
+      <c r="K1468">
+        <v>6670000</v>
+      </c>
+      <c r="L1468">
+        <v>6670000</v>
+      </c>
+    </row>
+    <row r="1469" spans="1:12">
+      <c r="A1469">
+        <v>1466</v>
+      </c>
+      <c r="B1469">
+        <v>403829</v>
+      </c>
+      <c r="C1469" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1469" t="s">
+        <v>1445</v>
+      </c>
+      <c r="E1469" t="s">
+        <v>1477</v>
+      </c>
+      <c r="F1469" t="s">
+        <v>1478</v>
+      </c>
+      <c r="G1469" t="s">
+        <v>1479</v>
+      </c>
+      <c r="H1469" t="s">
+        <v>272</v>
+      </c>
+      <c r="I1469" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1469">
+        <v>1</v>
+      </c>
+      <c r="K1469">
+        <v>1061323190</v>
+      </c>
+      <c r="L1469">
+        <v>1061323190</v>
+      </c>
+    </row>
+    <row r="1470" spans="1:12">
+      <c r="A1470">
+        <v>1467</v>
+      </c>
+      <c r="B1470">
+        <v>403829</v>
+      </c>
+      <c r="C1470" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1470" t="s">
+        <v>1445</v>
+      </c>
+      <c r="E1470" t="s">
+        <v>1480</v>
+      </c>
+      <c r="F1470" t="s">
+        <v>1481</v>
+      </c>
+      <c r="G1470" t="s">
+        <v>1482</v>
+      </c>
+      <c r="H1470" t="s">
+        <v>272</v>
+      </c>
+      <c r="I1470" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1470">
+        <v>1</v>
+      </c>
+      <c r="K1470">
+        <v>847674315</v>
+      </c>
+      <c r="L1470">
+        <v>847674315</v>
+      </c>
+    </row>
+    <row r="1471" spans="1:12">
+      <c r="A1471">
+        <v>1468</v>
+      </c>
+      <c r="B1471">
+        <v>403829</v>
+      </c>
+      <c r="C1471" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1471" t="s">
+        <v>1445</v>
+      </c>
+      <c r="E1471" t="s">
+        <v>1483</v>
+      </c>
+      <c r="F1471" t="s">
+        <v>1484</v>
+      </c>
+      <c r="G1471" t="s">
+        <v>1485</v>
+      </c>
+      <c r="H1471" t="s">
+        <v>233</v>
+      </c>
+      <c r="I1471" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1471">
+        <v>1</v>
+      </c>
+      <c r="K1471">
+        <v>2205000</v>
+      </c>
+      <c r="L1471">
+        <v>2205000</v>
+      </c>
+    </row>
+    <row r="1472" spans="1:12">
+      <c r="A1472">
+        <v>1469</v>
+      </c>
+      <c r="B1472">
+        <v>403829</v>
+      </c>
+      <c r="C1472" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1472" t="s">
+        <v>1445</v>
+      </c>
+      <c r="E1472" t="s">
+        <v>1483</v>
+      </c>
+      <c r="F1472" t="s">
+        <v>1484</v>
+      </c>
+      <c r="G1472" t="s">
+        <v>1485</v>
+      </c>
+      <c r="H1472" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1472" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1472">
+        <v>1</v>
+      </c>
+      <c r="K1472">
+        <v>23421000</v>
+      </c>
+      <c r="L1472">
+        <v>23421000</v>
+      </c>
+    </row>
+    <row r="1473" spans="1:12">
+      <c r="A1473">
+        <v>1470</v>
+      </c>
+      <c r="B1473">
+        <v>403829</v>
+      </c>
+      <c r="C1473" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1473" t="s">
+        <v>1445</v>
+      </c>
+      <c r="E1473" t="s">
+        <v>1486</v>
+      </c>
+      <c r="F1473" t="s">
+        <v>1487</v>
+      </c>
+      <c r="G1473" t="s">
+        <v>1488</v>
+      </c>
+      <c r="H1473" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1473" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1473">
+        <v>1</v>
+      </c>
+      <c r="K1473">
+        <v>218763054</v>
+      </c>
+      <c r="L1473">
+        <v>218763054</v>
+      </c>
+    </row>
+    <row r="1474" spans="1:12">
+      <c r="A1474">
+        <v>1471</v>
+      </c>
+      <c r="B1474">
+        <v>403829</v>
+      </c>
+      <c r="C1474" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1474" t="s">
+        <v>1445</v>
+      </c>
+      <c r="E1474" t="s">
+        <v>1489</v>
+      </c>
+      <c r="F1474" t="s">
+        <v>1490</v>
+      </c>
+      <c r="G1474" t="s">
+        <v>1491</v>
+      </c>
+      <c r="H1474" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1474" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1474">
+        <v>1</v>
+      </c>
+      <c r="K1474">
+        <v>287197847</v>
+      </c>
+      <c r="L1474">
+        <v>287197847</v>
+      </c>
+    </row>
+    <row r="1475" spans="1:12">
+      <c r="A1475">
+        <v>1472</v>
+      </c>
+      <c r="B1475">
+        <v>403829</v>
+      </c>
+      <c r="C1475" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1475" t="s">
+        <v>1445</v>
+      </c>
+      <c r="E1475" t="s">
+        <v>1492</v>
+      </c>
+      <c r="F1475" t="s">
+        <v>1493</v>
+      </c>
+      <c r="G1475" t="s">
+        <v>1494</v>
+      </c>
+      <c r="H1475" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1475" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1475">
+        <v>1</v>
+      </c>
+      <c r="K1475">
+        <v>157533431</v>
+      </c>
+      <c r="L1475">
+        <v>157533431</v>
+      </c>
+    </row>
+    <row r="1476" spans="1:12">
+      <c r="A1476">
+        <v>1473</v>
+      </c>
+      <c r="B1476">
+        <v>403829</v>
+      </c>
+      <c r="C1476" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1476" t="s">
+        <v>1445</v>
+      </c>
+      <c r="E1476" t="s">
+        <v>1495</v>
+      </c>
+      <c r="F1476" t="s">
+        <v>1496</v>
+      </c>
+      <c r="G1476" t="s">
+        <v>1497</v>
+      </c>
+      <c r="H1476" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1476" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1476">
+        <v>1</v>
+      </c>
+      <c r="K1476">
+        <v>102164682</v>
+      </c>
+      <c r="L1476">
+        <v>102164682</v>
+      </c>
+    </row>
+    <row r="1477" spans="1:12">
+      <c r="A1477">
+        <v>1474</v>
+      </c>
+      <c r="B1477">
+        <v>403829</v>
+      </c>
+      <c r="C1477" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1477" t="s">
+        <v>1498</v>
+      </c>
+      <c r="E1477" t="s">
+        <v>1499</v>
+      </c>
+      <c r="F1477" t="s">
+        <v>1500</v>
+      </c>
+      <c r="G1477" t="s">
+        <v>206</v>
+      </c>
+      <c r="H1477" t="s">
+        <v>1501</v>
+      </c>
+      <c r="I1477" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1477">
+        <v>1</v>
+      </c>
+      <c r="K1477">
+        <v>310000</v>
+      </c>
+      <c r="L1477">
+        <v>310000</v>
+      </c>
+    </row>
+    <row r="1478" spans="1:12">
+      <c r="A1478">
+        <v>1475</v>
+      </c>
+      <c r="B1478">
+        <v>403829</v>
+      </c>
+      <c r="C1478" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1478" t="s">
+        <v>1498</v>
+      </c>
+      <c r="E1478" t="s">
+        <v>1499</v>
+      </c>
+      <c r="F1478" t="s">
+        <v>1500</v>
+      </c>
+      <c r="G1478" t="s">
+        <v>206</v>
+      </c>
+      <c r="H1478" t="s">
+        <v>186</v>
+      </c>
+      <c r="I1478" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1478">
+        <v>1</v>
+      </c>
+      <c r="K1478">
+        <v>1000000</v>
+      </c>
+      <c r="L1478">
+        <v>1000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UP date realisasi per 5 Des 25
UP date realisasi per 5 Des 25
</commit_message>
<xml_diff>
--- a/Database/MONITORING DETAIL TRANSAKSI FA 16 SEGMEN VERSI SP2D.xlsx
+++ b/Database/MONITORING DETAIL TRANSAKSI FA 16 SEGMEN VERSI SP2D.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1783">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1790">
   <si>
     <t>MONITORING DETAIL TRANSAKSI FA 16 SEGMEN VERSI SP2D</t>
   </si>
@@ -5364,6 +5364,27 @@
   </si>
   <si>
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Nopember 2025 untuk 129 Pegawai</t>
+  </si>
+  <si>
+    <t>2025-12-05</t>
+  </si>
+  <si>
+    <t>'00523T</t>
+  </si>
+  <si>
+    <t>'259991320741000</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang berupa Tagihan PDAM Bulan Nopember 2025 Idple No. 1249-1046 An Lemb Perikanan Darat</t>
+  </si>
+  <si>
+    <t>'00524T</t>
+  </si>
+  <si>
+    <t>'259991311304509</t>
+  </si>
+  <si>
+    <t>'403829.023.523121.03212WA.2378EBA.A000000001.00000.2.0252.2.000000.000000.994.002.DC.000305</t>
   </si>
 </sst>
 </file>
@@ -5706,7 +5727,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:L1798"/>
+  <dimension ref="A1:L1811"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -73961,6 +73982,500 @@
       </c>
       <c r="L1798">
         <v>11060000</v>
+      </c>
+    </row>
+    <row r="1799" spans="1:12">
+      <c r="A1799">
+        <v>1796</v>
+      </c>
+      <c r="B1799">
+        <v>403829</v>
+      </c>
+      <c r="C1799" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1799" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1799" t="s">
+        <v>1784</v>
+      </c>
+      <c r="F1799" t="s">
+        <v>1785</v>
+      </c>
+      <c r="G1799" t="s">
+        <v>1786</v>
+      </c>
+      <c r="H1799" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1799" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1799">
+        <v>1</v>
+      </c>
+      <c r="K1799">
+        <v>604300</v>
+      </c>
+      <c r="L1799">
+        <v>604300</v>
+      </c>
+    </row>
+    <row r="1800" spans="1:12">
+      <c r="A1800">
+        <v>1797</v>
+      </c>
+      <c r="B1800">
+        <v>403829</v>
+      </c>
+      <c r="C1800" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1800" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1800" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1800" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1800" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1800" t="s">
+        <v>173</v>
+      </c>
+      <c r="I1800" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1800">
+        <v>1</v>
+      </c>
+      <c r="K1800">
+        <v>3953112</v>
+      </c>
+      <c r="L1800">
+        <v>3953112</v>
+      </c>
+    </row>
+    <row r="1801" spans="1:12">
+      <c r="A1801">
+        <v>1798</v>
+      </c>
+      <c r="B1801">
+        <v>403829</v>
+      </c>
+      <c r="C1801" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1801" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1801" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1801" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1801" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1801" t="s">
+        <v>1584</v>
+      </c>
+      <c r="I1801" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1801">
+        <v>1</v>
+      </c>
+      <c r="K1801">
+        <v>50601600</v>
+      </c>
+      <c r="L1801">
+        <v>50601600</v>
+      </c>
+    </row>
+    <row r="1802" spans="1:12">
+      <c r="A1802">
+        <v>1799</v>
+      </c>
+      <c r="B1802">
+        <v>403829</v>
+      </c>
+      <c r="C1802" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1802" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1802" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1802" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1802" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1802" t="s">
+        <v>386</v>
+      </c>
+      <c r="I1802" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1802">
+        <v>1</v>
+      </c>
+      <c r="K1802">
+        <v>300000</v>
+      </c>
+      <c r="L1802">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="1803" spans="1:12">
+      <c r="A1803">
+        <v>1800</v>
+      </c>
+      <c r="B1803">
+        <v>403829</v>
+      </c>
+      <c r="C1803" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1803" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1803" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1803" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1803" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1803" t="s">
+        <v>159</v>
+      </c>
+      <c r="I1803" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1803">
+        <v>1</v>
+      </c>
+      <c r="K1803">
+        <v>180000</v>
+      </c>
+      <c r="L1803">
+        <v>180000</v>
+      </c>
+    </row>
+    <row r="1804" spans="1:12">
+      <c r="A1804">
+        <v>1801</v>
+      </c>
+      <c r="B1804">
+        <v>403829</v>
+      </c>
+      <c r="C1804" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1804" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1804" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1804" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1804" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1804" t="s">
+        <v>174</v>
+      </c>
+      <c r="I1804" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1804">
+        <v>1</v>
+      </c>
+      <c r="K1804">
+        <v>1380500</v>
+      </c>
+      <c r="L1804">
+        <v>1380500</v>
+      </c>
+    </row>
+    <row r="1805" spans="1:12">
+      <c r="A1805">
+        <v>1802</v>
+      </c>
+      <c r="B1805">
+        <v>403829</v>
+      </c>
+      <c r="C1805" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1805" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1805" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1805" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1805" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1805" t="s">
+        <v>178</v>
+      </c>
+      <c r="I1805" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1805">
+        <v>1</v>
+      </c>
+      <c r="K1805">
+        <v>9468528</v>
+      </c>
+      <c r="L1805">
+        <v>9468528</v>
+      </c>
+    </row>
+    <row r="1806" spans="1:12">
+      <c r="A1806">
+        <v>1803</v>
+      </c>
+      <c r="B1806">
+        <v>403829</v>
+      </c>
+      <c r="C1806" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1806" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1806" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1806" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1806" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1806" t="s">
+        <v>1710</v>
+      </c>
+      <c r="I1806" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1806">
+        <v>1</v>
+      </c>
+      <c r="K1806">
+        <v>22953312</v>
+      </c>
+      <c r="L1806">
+        <v>22953312</v>
+      </c>
+    </row>
+    <row r="1807" spans="1:12">
+      <c r="A1807">
+        <v>1804</v>
+      </c>
+      <c r="B1807">
+        <v>403829</v>
+      </c>
+      <c r="C1807" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1807" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1807" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1807" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1807" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1807" t="s">
+        <v>1711</v>
+      </c>
+      <c r="I1807" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1807">
+        <v>1</v>
+      </c>
+      <c r="K1807">
+        <v>4629928</v>
+      </c>
+      <c r="L1807">
+        <v>4629928</v>
+      </c>
+    </row>
+    <row r="1808" spans="1:12">
+      <c r="A1808">
+        <v>1805</v>
+      </c>
+      <c r="B1808">
+        <v>403829</v>
+      </c>
+      <c r="C1808" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1808" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1808" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1808" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1808" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1808" t="s">
+        <v>185</v>
+      </c>
+      <c r="I1808" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1808">
+        <v>1</v>
+      </c>
+      <c r="K1808">
+        <v>2890000</v>
+      </c>
+      <c r="L1808">
+        <v>2890000</v>
+      </c>
+    </row>
+    <row r="1809" spans="1:12">
+      <c r="A1809">
+        <v>1806</v>
+      </c>
+      <c r="B1809">
+        <v>403829</v>
+      </c>
+      <c r="C1809" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1809" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1809" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1809" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1809" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1809" t="s">
+        <v>186</v>
+      </c>
+      <c r="I1809" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1809">
+        <v>1</v>
+      </c>
+      <c r="K1809">
+        <v>1490000</v>
+      </c>
+      <c r="L1809">
+        <v>1490000</v>
+      </c>
+    </row>
+    <row r="1810" spans="1:12">
+      <c r="A1810">
+        <v>1807</v>
+      </c>
+      <c r="B1810">
+        <v>403829</v>
+      </c>
+      <c r="C1810" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1810" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1810" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1810" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1810" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1810" t="s">
+        <v>191</v>
+      </c>
+      <c r="I1810" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1810">
+        <v>1</v>
+      </c>
+      <c r="K1810">
+        <v>1560138</v>
+      </c>
+      <c r="L1810">
+        <v>1560138</v>
+      </c>
+    </row>
+    <row r="1811" spans="1:12">
+      <c r="A1811">
+        <v>1808</v>
+      </c>
+      <c r="B1811">
+        <v>403829</v>
+      </c>
+      <c r="C1811" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1811" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E1811" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F1811" t="s">
+        <v>1788</v>
+      </c>
+      <c r="G1811" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1811" t="s">
+        <v>1789</v>
+      </c>
+      <c r="I1811" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1811">
+        <v>1</v>
+      </c>
+      <c r="K1811">
+        <v>750000</v>
+      </c>
+      <c r="L1811">
+        <v>750000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>